<commit_message>
Uitgebreide feedbackronde: 5 nieuwe RULES.md-regels, De Keuken van Sandra eruit
Nieuwe permanente regels (elk bevestigd op meerdere sites): verbod op
scroll-voortgangsbalk, nooit twee header-links naar dezelfde pagina,
nieuwe sectie Grid- en kaartlayouts met voorkeur voor symmetrie boven
asymmetrische bento-grids, verplichte scherpte-check op foto's, en
pitchmails moeten voortaan concrete klantwaarde (SEO/vindbaarheid)
benoemen.

De Keuken van Sandra is op verzoek van Sem uit companies.json en pitches/
verwijderd; de GitHub-repo zelf moet handmatig verwijderd worden (geen
tool hiervoor beschikbaar).
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -170,8 +170,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:L5" headerRowCount="1">
-  <autoFilter ref="A1:L5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:L4" headerRowCount="1">
+  <autoFilter ref="A1:L4"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -744,68 +744,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>De Keuken van Sandra</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Sandra Kaag</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Catering, workshops, patisserie en lunches aan huis (foodstyling/culinair)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Wateringen / Westland / Den Haag</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>dekeukenvansandra</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/dekeukenvansandra/</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>06 27 49 50 01</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>sandra@dekeukenvansandra.nl</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Intake: Cone6 toegevoegd aan wachtrij (issue #1)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
         <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5E7EB"/>
+        <bgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -91,6 +97,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -170,8 +179,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:L4" headerRowCount="1">
-  <autoFilter ref="A1:L4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:L6" headerRowCount="1">
+  <autoFilter ref="A1:L6"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -479,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -744,6 +753,114 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cone6</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Yvonne da Silva</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Keramiekatelier (workshops, cursussen, teambuilding, stookservice)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Den Hoorn / Den Haag Zuid / Westland / Delft</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>cone6</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>06 244 606 96</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>cone6keramiek@gmail.com</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Angelina de Jong</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Dierenkliniek / dierenarts (honden, katten, konijnen, knaagdieren)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Delft (Harnaschpolder)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>dierenkliniek-animalis</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>015 737 0135</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>dierenarts@dierenkliniekanimalis.nl</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
NIEUWE BUILD: Cone6 en Dierenkliniek Animalis opgepakt
Blok 1 (17:00), volledig nachtbudget (2/2 builds).
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -57,8 +57,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E5E7EB"/>
-        <bgColor rgb="00E5E7EB"/>
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -776,7 +776,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Cone6 + Dierenkliniek Animalis terug naar pending (bouw onderbroken)
Beide bouw-subagents werden in blok 1 vrijwel meteen na de start
onverwacht gestopt (status "killed"), voordat er enige site-code
geschreven was. Beide doel-repo's bevestigd nog leeg, dus geen
verloren werk. Terug naar status pending zodat een volgend blok het
gewoon opnieuw kan oppakken.
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -57,8 +57,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00E5E7EB"/>
+        <bgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -776,7 +776,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Cone6 en Dierenkliniek Animalis hervat
Sem's 5-uursvenster is ververst, ze heeft expliciet gevraagd de eerder
onderbroken bouwpogingen nu te hervatten.
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -57,8 +57,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E5E7EB"/>
-        <bgColor rgb="00E5E7EB"/>
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -776,7 +776,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dierenkliniek Animalis: site gebouwd, needs_review (deploy-check)
Site volledig gebouwd en gecontroleerd (acht-staps kwaliteitscontrole),
conceptpitchmail klaar in pitches/dierenkliniek-animalis.md. Status
needs_review: de Pages-deploy kon nog niet bevestigd worden groen na
de bekende race-condition op een gloednieuwe repo, reden en
vervolgstappen staan in de notities.
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
         <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -100,6 +106,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -828,9 +837,9 @@
           <t>Delft (Harnaschpolder)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -838,10 +847,14 @@
           <t>dierenkliniek-animalis</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/ (deploy nog niet bevestigd groen, zie notities)</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Cone6: site gebouwd, needs_review (deploy-check)
Site volledig gebouwd, getest en gepusht (NL/EN, aparte FAQ- en
voorwaardenpagina, teambuilding met echte klantlogo's). Conceptpitchmail
klaar in pitches/cone6.md. Status needs_review: net als
dierenkliniek-animalis faalde de Pages-deploy op de "Setup Pages"-stap
zonder automatisch herstel. Twee gloednieuwe repo's op dezelfde avond
met exact dezelfde fout wijst op iets structureels, zie notities voor
een mogelijke oorzaak (Pages-instelling per repo).
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,12 +53,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
         <bgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -106,9 +100,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -785,7 +776,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -793,10 +784,14 @@
           <t>cone6</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/cone6/ (deploy nog niet bevestigd groen, zie notities)</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -837,7 +832,7 @@
           <t>Delft (Harnaschpolder)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>needs_review</t>
         </is>

</xml_diff>

<commit_message>
Cone6 + Dierenkliniek Animalis: deploy bevestigd, status naar done
Sem zette Settings > Pages > Source handmatig op 'GitHub Actions' voor
beide gloednieuwe repo's (de structurele oorzaak van de eerdere
deploy-fout), reruns bevestigd succesvol voor beide.
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,12 +53,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
         <bgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
-        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -97,9 +91,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -774,9 +765,9 @@
           <t>Den Hoorn / Den Haag Zuid / Westland / Delft</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -786,7 +777,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cone6/ (deploy nog niet bevestigd groen, zie notities)</t>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -809,7 +800,11 @@
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -832,9 +827,9 @@
           <t>Delft (Harnaschpolder)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -844,7 +839,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/ (deploy nog niet bevestigd groen, zie notities)</t>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -867,7 +862,11 @@
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Verzendstatus pitchmail toevoegen aan companies.json en overzicht.xlsx
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
         <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -91,6 +97,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -170,9 +179,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:L6" headerRowCount="1">
-  <autoFilter ref="A1:L6"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:N6" headerRowCount="1">
+  <autoFilter ref="A1:N6"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
     <tableColumn id="3" name="Branche"/>
@@ -181,10 +190,12 @@
     <tableColumn id="6" name="Repo"/>
     <tableColumn id="7" name="Live URL"/>
     <tableColumn id="8" name="Pitchmail klaar"/>
-    <tableColumn id="9" name="Telefoon"/>
-    <tableColumn id="10" name="E-mail"/>
-    <tableColumn id="11" name="Toegevoegd op"/>
-    <tableColumn id="12" name="Afgerond op"/>
+    <tableColumn id="9" name="Pitchmail verzonden"/>
+    <tableColumn id="10" name="Verzonden op"/>
+    <tableColumn id="11" name="Telefoon"/>
+    <tableColumn id="12" name="E-mail"/>
+    <tableColumn id="13" name="Toegevoegd op"/>
+    <tableColumn id="14" name="Afgerond op"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
 </table>
@@ -479,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -491,9 +502,11 @@
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -539,20 +552,30 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Pitchmail verzonden</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Verzonden op</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Telefoon</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Toegevoegd op</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Afgerond op</t>
         </is>
@@ -599,22 +622,28 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>06-81502169</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>info@ziehaarstralen.nl</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
@@ -661,22 +690,28 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>015-2120610</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>info@vanoostenvoorvis.nl</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
@@ -723,22 +758,32 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>06 23 774 773</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>info@manimania.nl</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
@@ -785,22 +830,28 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>06 244 606 96</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>cone6keramiek@gmail.com</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
@@ -847,22 +898,28 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>015 737 0135</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>dierenarts@dierenkliniekanimalis.nl</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>

</xml_diff>

<commit_message>
Cone6: pitchmail verstuurd (28-07-2026)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -830,12 +830,16 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
           <t>06 244 606 96</t>

</xml_diff>

<commit_message>
Van Oosten voor Vis: pitchmail verstuurd (27-07-2026)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -690,12 +690,16 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
           <t>015-2120610</t>

</xml_diff>

<commit_message>
Dierenkliniek Animalis: pitchmail verstuurd (28-07-2026)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -906,12 +906,16 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
           <t>015 737 0135</t>

</xml_diff>

<commit_message>
Klantreactie + follow-up-datum toevoegen aan companies.json en overzicht.xlsx
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
         <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5E7EB"/>
+        <bgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -100,6 +106,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -179,9 +188,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:N6" headerRowCount="1">
-  <autoFilter ref="A1:N6"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P6" headerRowCount="1">
+  <autoFilter ref="A1:P6"/>
+  <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
     <tableColumn id="3" name="Branche"/>
@@ -192,10 +201,12 @@
     <tableColumn id="8" name="Pitchmail klaar"/>
     <tableColumn id="9" name="Pitchmail verzonden"/>
     <tableColumn id="10" name="Verzonden op"/>
-    <tableColumn id="11" name="Telefoon"/>
-    <tableColumn id="12" name="E-mail"/>
-    <tableColumn id="13" name="Toegevoegd op"/>
-    <tableColumn id="14" name="Afgerond op"/>
+    <tableColumn id="11" name="Klantreactie"/>
+    <tableColumn id="12" name="Follow-up op"/>
+    <tableColumn id="13" name="Telefoon"/>
+    <tableColumn id="14" name="E-mail"/>
+    <tableColumn id="15" name="Toegevoegd op"/>
+    <tableColumn id="16" name="Afgerond op"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
 </table>
@@ -490,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -503,10 +514,12 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -562,20 +575,30 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Klantreactie</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Follow-up op</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Telefoon</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Toegevoegd op</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Afgerond op</t>
         </is>
@@ -628,22 +651,28 @@
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>06-81502169</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>info@ziehaarstralen.nl</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
@@ -700,22 +729,28 @@
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>015-2120610</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>info@vanoostenvoorvis.nl</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
@@ -772,22 +807,28 @@
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>06 23 774 773</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>info@manimania.nl</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
@@ -844,22 +885,28 @@
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>06 244 606 96</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>cone6keramiek@gmail.com</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
@@ -916,22 +963,28 @@
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>015 737 0135</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>dierenarts@dierenkliniekanimalis.nl</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>

</xml_diff>

<commit_message>
Intake: BitWizard B.V. toegevoegd aan wachtrij (issue #4)
Intake: Meijer Administratieve Diensten toegevoegd aan wachtrij (issue #5)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P6" headerRowCount="1">
-  <autoFilter ref="A1:P6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P8" headerRowCount="1">
+  <autoFilter ref="A1:P8"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -990,6 +990,126 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Elektronica-/IT-ingenieursbedrijf (custom elektronicaontwikkeling, Linux-diensten, netwerkdiensten, webshop met Raspberry Pi/Arduino-uitbreidingsborden)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Delfgauw (tussen Den Haag en Rotterdam, bij de A13)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>bitwizard-demo</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>+31 (0)15-2049110</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Meijer Administratieve Diensten</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Administratiekantoor / boekhouder (financiële administratie, loonadministratie, belastingaangiften voor bedrijven en particulieren)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Delft / Rotterdam / Den Haag / Westland</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>meijer-administratievediensten-demo</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>015 - 2 13 23 03</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>info@meijerad.nl</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
NIEUWE BUILD: BitWizard B.V. opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1007,9 +1007,9 @@
           <t>Delfgauw (tussen Den Haag en Rotterdam, bij de A13)</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
BitWizard B.V.: site gebouwd en live (commit b576436), conceptpitchmail klaar
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1007,9 +1007,9 @@
           <t>Delfgauw (tussen Den Haag en Rotterdam, bij de A13)</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1017,13 +1017,17 @@
           <t>bitwizard-demo</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -1046,7 +1050,11 @@
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Meijer Administratieve Diensten opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1073,9 +1073,9 @@
           <t>Delft / Rotterdam / Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Meijer Administratieve Diensten: build tweemaal mislukt op 529 Overloaded, terug naar pending; PIPELINE.md: onderscheid infra-fout vs. inhoudelijk probleem
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1073,9 +1073,9 @@
           <t>Delft / Rotterdam / Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Meijer Administratieve Diensten opnieuw opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1073,9 +1073,9 @@
           <t>Delft / Rotterdam / Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Nachtrun 30-07: wekelijkse limiet bereikt, BitWizard-feedback en Meijer-build teruggezet voor volgende run
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1073,9 +1073,9 @@
           <t>Delft / Rotterdam / Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Meijer Administratieve Diensten opnieuw opgepakt (na wekelijkse limiet-reset)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1073,9 +1073,9 @@
           <t>Delft / Rotterdam / Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Meijer-build handmatig gestopt door Sem, teruggezet naar pending voor de nachtelijke run
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1073,9 +1073,9 @@
           <t>Delft / Rotterdam / Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Intake: Cocon toegevoegd aan wachtrij (issue #8)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P8" headerRowCount="1">
-  <autoFilter ref="A1:P8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P9" headerRowCount="1">
+  <autoFilter ref="A1:P9"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1118,6 +1118,64 @@
       </c>
       <c r="P8" s="2" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Cocon</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ditte Wismeyer en Michael Dijkhuizen</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Bed &amp; Breakfast met culinaire gastvrijheid (gastenverblijf in oprichting, nog geen definitieve locatie)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Limburg / Heuvelland (o.a. Gulpen)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>cocon-b-b-demo</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Meijer Administratieve Diensten: build succesvol, status done, pitchmail klaar
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1073,9 +1073,9 @@
           <t>Delft / Rotterdam / Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1083,13 +1083,17 @@
           <t>meijer-administratievediensten-demo</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -1116,7 +1120,11 @@
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Cocon opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1147,9 +1147,9 @@
           <t>Zuid-Limburg / Heuvelland (o.a. Gulpen)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Cocon: build succesvol, status done, pitchmail klaar
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1147,9 +1147,9 @@
           <t>Zuid-Limburg / Heuvelland (o.a. Gulpen)</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1157,13 +1157,17 @@
           <t>cocon-b-b</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -1182,7 +1186,11 @@
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Intake: Smithuis Installatiebedrijf toegevoegd aan wachtrij (issue #12)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P9" headerRowCount="1">
-  <autoFilter ref="A1:P9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P10" headerRowCount="1">
+  <autoFilter ref="A1:P10"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1192,6 +1192,72 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Smithuis Installatiebedrijf</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Michael Smithuis</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Installatietechniek / allround klusbedrijf (CV-ketels, water/gas/sanitair, badkamers, zonnepanelen, elektra, klein bouwkundig werk)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Delft e.o. (Zuid-Holland; klanten o.a. uit Rotterdam, Den Haag, Schiedam, Zoetermeer, Vlaardingen)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>smithuis-installatie</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>06 23800848</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>smithuisinstallatie@hotmail.com</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
NIEUWE BUILD: Smithuis Installatiebedrijf opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1213,9 +1213,9 @@
           <t>Delft e.o. (Zuid-Holland; klanten o.a. uit Rotterdam, Den Haag, Schiedam, Zoetermeer, Vlaardingen)</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Smithuis Installatiebedrijf: build succesvol afgerond, pitchmail klaar
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1213,9 +1213,9 @@
           <t>Delft e.o. (Zuid-Holland; klanten o.a. uit Rotterdam, Den Haag, Schiedam, Zoetermeer, Vlaardingen)</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1223,13 +1223,17 @@
           <t>smithuis-installatie</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -1256,7 +1260,11 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
BitWizard: pitchmail verstuurd (04-08-2026)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1027,12 +1027,16 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
           <t>nog geen reactie</t>

</xml_diff>

<commit_message>
Intake: Schilperoort IJzerwaren toegevoegd aan wachtrij (issue #14)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P10" headerRowCount="1">
-  <autoFilter ref="A1:P10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P11" headerRowCount="1">
+  <autoFilter ref="A1:P11"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1270,6 +1270,72 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Schilperoort IJzerwaren</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Onno Schilperoort en Remco Schilperoort</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>IJzerwarenwinkel (sleutelservice, verlichting, gereedschappen, verf, tuinartikelen, naambordjes)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Rijswijk</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>schilderpoort-ijzerwaren</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>070-3935325 (Bogaard) / 070-3954117 (Herenstraat)</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>bogaard@schilperoort-ijzerwaren.nl / herenstraat@schilperoort-ijzerwaren.nl</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Intake: Wisselbekers toegevoegd aan wachtrij (issue #16)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P12" headerRowCount="1">
-  <autoFilter ref="A1:P12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P13" headerRowCount="1">
+  <autoFilter ref="A1:P13"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1398,6 +1398,64 @@
       </c>
       <c r="P12" s="2" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Wisselbekers</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Duurzaam retour-/recyclingsysteem voor kartonnen koffiebekers (B2B, initiatief van Wildenberg Recycling)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Den Haag</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>070-5113662</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>info@wisselbekers.nl</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Intake: Garagebedrijf Dennis toegevoegd aan wachtrij (issue #15)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P11" headerRowCount="1">
-  <autoFilter ref="A1:P11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P12" headerRowCount="1">
+  <autoFilter ref="A1:P12"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1336,6 +1336,68 @@
       </c>
       <c r="P11" s="2" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Garagebedrijf Dennis</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Dennis</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Autogarage / RDW-erkend APK-keuringsstation (reparaties, onderhoud, alle merken)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Den Haag</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>garagebedrijf-dennis</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>070-3080596 / 06-16724822</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Intake: Geo B.V. toegevoegd aan wachtrij (issue #17)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P13" headerRowCount="1">
-  <autoFilter ref="A1:P13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P14" headerRowCount="1">
+  <autoFilter ref="A1:P14"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1456,6 +1456,68 @@
       </c>
       <c r="P13" s="2" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Oliehandel / bunkerbedrijf (gasolie, smeeroliën, scheepsbenodigdheden) voor visserij, zeevaart, offshore en binnenvaart</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Barendrecht / Stellendam / Scheveningen (Zuid-Holland, havens en scheepvaart)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>nog geen reactie</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>078-6772682 (kantoor Barendrecht) / 06-53487162 (bunkerboot Stellendam) / 06-25593581 (bunkerboot Scheveningen)</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>info@geobv.nl</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
NIEUWE BUILD: Schilperoort IJzerwaren opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1291,9 +1291,9 @@
           <t>Rijswijk</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Schilperoort IJzerwaren: bouwpoging mislukt op account-uitgavenlimiet, terug naar pending
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1291,9 +1291,9 @@
           <t>Rijswijk</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Schilperoort IJzerwaren opgepakt (poging 2)
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1291,9 +1291,9 @@
           <t>Rijswijk</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Schilperoort IJzerwaren: vastgelopen in_progress (29u, BLOK BOUW vuurde niet), naar needs_review
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
         <bgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -94,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -109,6 +115,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1291,9 +1300,9 @@
           <t>Rijswijk</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Garagebedrijf Dennis opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1366,9 +1366,9 @@
           <t>Den Haag</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Garagebedrijf Dennis: build afgerond, pitchmail toegevoegd
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1366,9 +1366,9 @@
           <t>Den Haag</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1376,13 +1376,17 @@
           <t>garagebedrijf-dennis</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -1405,7 +1409,11 @@
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
NIEUWE BUILD: Geo B.V. opgepakt
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1490,9 +1490,9 @@
           <t>Barendrecht / Stellendam / Scheveningen (Zuid-Holland, havens en scheepvaart)</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Geo B.V.: build afgerond, pitchmail toegevoegd
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -1490,9 +1490,9 @@
           <t>Barendrecht / Stellendam / Scheveningen (Zuid-Holland, havens en scheepvaart)</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>in_progress</t>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1500,13 +1500,17 @@
           <t>geo</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -1533,7 +1537,11 @@
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Overzicht: updategeschiedenis per site (wanneer + wat aangepast)
Op verzoek van Sem: overzicht.xlsx toont nu per site wanneer die is gebouwd of
aangepast en wat er veranderd is, zodat ze makkelijk kan controleren.

- companies.json: nieuw 'updates'-veld per bedrijf (lijst met datum/wat/commit/
  live_url), met accurate backfill uit de bestaande notities.
- generate_overzicht.py: hoofdtab toont 'Laatste update' + 'Laatste wijziging';
  nieuwe tab 'Updategeschiedenis' met alle wijzigingen chronologisch (nieuwste
  eerst).
- PIPELINE.md: BLOK BOUW (succes) en BLOK FEEDBACK loggen voortaan een
  updates-entry en verversen het overzicht.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Overzicht" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Updategeschiedenis" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -117,8 +118,17 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -197,9 +207,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:P14" headerRowCount="1">
-  <autoFilter ref="A1:P14"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BedrijvenOverzicht" displayName="BedrijvenOverzicht" ref="A1:R14" headerRowCount="1">
+  <autoFilter ref="A1:R14"/>
+  <tableColumns count="18">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Contactpersoon"/>
     <tableColumn id="3" name="Branche"/>
@@ -216,6 +226,22 @@
     <tableColumn id="14" name="E-mail"/>
     <tableColumn id="15" name="Toegevoegd op"/>
     <tableColumn id="16" name="Afgerond op"/>
+    <tableColumn id="17" name="Laatste update"/>
+    <tableColumn id="18" name="Laatste wijziging"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E19" headerRowCount="1">
+  <autoFilter ref="A1:E19"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Bedrijfsnaam"/>
+    <tableColumn id="2" name="Datum"/>
+    <tableColumn id="3" name="Wat is er veranderd"/>
+    <tableColumn id="4" name="Commit"/>
+    <tableColumn id="5" name="Live URL"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showRowStripes="1"/>
 </table>
@@ -510,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -529,6 +555,8 @@
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -612,6 +640,16 @@
           <t>Afgerond op</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Laatste update</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Laatste wijziging</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -686,6 +724,16 @@
           <t>2026-07-23</t>
         </is>
       </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -764,6 +812,16 @@
           <t>2026-07-24</t>
         </is>
       </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -842,6 +900,16 @@
           <t>2026-07-25</t>
         </is>
       </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>Feedbackronde: echte prijslijst verwerkt in nieuwe prijzen.html, 5 extra foto's opnieuw geplaatst, regio gecorrigeerd</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -920,6 +988,16 @@
           <t>2026-07-27</t>
         </is>
       </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>Feedbackronde: kaarten gelijk gemaakt, bannercontrast, logo bijgesneden, logo-marquee doorlopend; mailto hersteld en verboden tekst verwijderd</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -998,6 +1076,16 @@
           <t>2026-07-27</t>
         </is>
       </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1068,6 +1156,16 @@
           <t>2026-07-28</t>
         </is>
       </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1136,6 +1234,16 @@
       <c r="P8" s="2" t="inlineStr">
         <is>
           <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
         </is>
       </c>
     </row>
@@ -1204,6 +1312,16 @@
           <t>2026-08-01</t>
         </is>
       </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1278,6 +1396,16 @@
           <t>2026-08-04</t>
         </is>
       </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1300,7 +1428,7 @@
           <t>Rijswijk</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>needs_review</t>
         </is>
@@ -1344,6 +1472,16 @@
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN-taalswitcher, beeldmateriaal, taal/menu-polish) maar niet afgerond; op needs_review gezet</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1412,6 +1550,16 @@
       <c r="P12" s="2" t="inlineStr">
         <is>
           <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
         </is>
       </c>
     </row>
@@ -1472,6 +1620,8 @@
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1540,6 +1690,513 @@
       <c r="P14" s="2" t="inlineStr">
         <is>
           <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bedrijfsnaam</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Wat is er veranderd</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Live URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr"/>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Schilperoort IJzerwaren</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN-taalswitcher, beeldmateriaal, taal/menu-polish) maar niet afgerond; op needs_review gezet</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr"/>
+      <c r="E3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Garagebedrijf Dennis</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr"/>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Smithuis Installatiebedrijf</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>c749bd4</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Cocon</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>b42a083</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Meijer Administratieve Diensten</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Cone6</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Feedbackronde: kaarten gelijk gemaakt, bannercontrast, logo bijgesneden, logo-marquee doorlopend; mailto hersteld en verboden tekst verwijderd</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>eb2a9c7</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Tweede feedbackronde: VetPlan-knop/disclaimer herzien, contactformulier-melding na klik, kaart-uitlijning, hamburgermenu-bugs</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>5ce93c69</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>716874d</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>b576436</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>ManiMania</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Feedbackronde: echte prijslijst verwerkt in nieuwe prijzen.html, 5 extra foto's opnieuw geplaatst, regio gecorrigeerd</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Cone6</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>a5daae7</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>2c24e39</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Feedbackronde: echt logo verwerkt, openingstijden per dag, diersoort-iconen opnieuw getekend, mobiele overflow-fix</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>0e586ac</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>ManiMania</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Van Oosten voor Vis</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr"/>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Zie Haar Stralen</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Overzicht/pipeline: bullets, done pas na akkoord, pitchmail meebewerken, datum dd-mm-jjjj
Op verzoek van Sem (18-08-2026):
- Wijzigingen als losse '-'-puntjes onder elkaar (wat-veld is nu een lijst).
- Nieuwe status 'wacht_op_akkoord': een gebouwde site krijgt niet meer
  automatisch 'done'; done pas als Sem mailt of akkoord geeft. 6 bestaande,
  nog-niet-gemailde sites teruggezet naar wacht_op_akkoord.
- BLOK FEEDBACK werkt voortaan ook de pitchmail bij als feedback iets raakt
  wat in de pitch staat (bijv. extra taal).
- Overzicht toont datums altijd als dd-mm-jjjj (intern blijft JJJJ-MM-DD voor
  sortering).
- Footer-retrofit en compliance-sweep tellen nu done + wacht_op_akkoord als
  live site.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -37,7 +37,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +52,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
-        <bgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -66,6 +66,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E5E7EB"/>
         <bgColor rgb="00E5E7EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,16 +125,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -543,7 +549,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -674,7 +680,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>Wacht op akkoord</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -716,22 +722,22 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="R2" s="6" t="inlineStr">
         <is>
-          <t>Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
     </row>
@@ -756,9 +762,9 @@
           <t>Delft</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -776,14 +782,14 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -804,22 +810,22 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="R3" s="6" t="inlineStr">
         <is>
-          <t>Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
     </row>
@@ -844,9 +850,9 @@
           <t>Den Haag / Westland</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -864,14 +870,14 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -892,22 +898,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
         <is>
-          <t>Feedbackronde: echte prijslijst verwerkt in nieuwe prijzen.html, 5 extra foto's opnieuw geplaatst, regio gecorrigeerd</t>
+          <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
+- 5 extra foto's opnieuw geplaatst
+- Regio gecorrigeerd</t>
         </is>
       </c>
     </row>
@@ -932,9 +940,9 @@
           <t>Den Hoorn / Den Haag Zuid / Westland / Delft</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -952,14 +960,14 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -980,22 +988,25 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t>Feedbackronde: kaarten gelijk gemaakt, bannercontrast, logo bijgesneden, logo-marquee doorlopend; mailto hersteld en verboden tekst verwijderd</t>
+          <t>- Kaarten op gelijke hoogte gebracht
+- Bannercontrast verbeterd
+- Logo bijgesneden en logo-marquee doorlopend gemaakt
+- Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
     </row>
@@ -1020,9 +1031,9 @@
           <t>Delft (Harnaschpolder)</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1040,14 +1051,14 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1068,22 +1079,22 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
         <is>
-          <t>Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
         </is>
       </c>
     </row>
@@ -1104,9 +1115,9 @@
           <t>Delfgauw (tussen Den Haag en Rotterdam, bij de A13)</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1124,14 +1135,14 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1148,22 +1159,22 @@
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>30-07-2026</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
         <is>
-          <t>Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1197,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>Wacht op akkoord</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1228,22 +1239,22 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1281,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>Wacht op akkoord</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1304,22 +1315,22 @@
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
         <is>
-          <t>Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1357,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>Wacht op akkoord</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1388,22 +1399,22 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>03-08-2026</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
         <is>
-          <t>Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
     </row>
@@ -1428,9 +1439,9 @@
           <t>Rijswijk</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Needs review</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1468,18 +1479,19 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
         <is>
-          <t>Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN-taalswitcher, beeldmateriaal, taal/menu-polish) maar niet afgerond; op needs_review gezet</t>
+          <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
+- Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1518,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>Wacht op akkoord</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1544,22 +1556,22 @@
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
         <is>
-          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1594,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="F13" s="2" t="n"/>
@@ -1616,7 +1628,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr"/>
@@ -1642,7 +1654,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>Wacht op akkoord</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1684,22 +1696,22 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
         <is>
-          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
         </is>
       </c>
     </row>
@@ -1755,446 +1767,458 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Geo B.V.</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="inlineStr"/>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr"/>
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN-taalswitcher, beeldmateriaal, taal/menu-polish) maar niet afgerond; op needs_review gezet</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr"/>
-      <c r="E3" s="8" t="inlineStr"/>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
+- Niet afgerond; op needs_review gezet</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr"/>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>10-08-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>04-08-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>c749bd4</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Cocon</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>01-08-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>b42a083</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr"/>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>31-07-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>BitWizard B.V.</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr"/>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Feedbackronde: kaarten gelijk gemaakt, bannercontrast, logo bijgesneden, logo-marquee doorlopend; mailto hersteld en verboden tekst verwijderd</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>- Kaarten op gelijke hoogte gebracht
+- Bannercontrast verbeterd
+- Logo bijgesneden en logo-marquee doorlopend gemaakt
+- Mailto-verzending hersteld en verboden tekst verwijderd</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Tweede feedbackronde: VetPlan-knop/disclaimer herzien, contactformulier-melding na klik, kaart-uitlijning, hamburgermenu-bugs</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>- VetPlan-knop en -disclaimer herzien
+- Contactformulier-melding pas na klik
+- Kaart-uitlijning gecorrigeerd
+- Hamburgermenu-bugs opgelost</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>5ce93c69</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>716874d</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>BitWizard B.V.</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>b576436</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Feedbackronde: echte prijslijst verwerkt in nieuwe prijzen.html, 5 extra foto's opnieuw geplaatst, regio gecorrigeerd</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr"/>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
+- 5 extra foto's opnieuw geplaatst
+- Regio gecorrigeerd</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr"/>
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>a5daae7</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>2c24e39</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Feedbackronde: echt logo verwerkt, openingstijden per dag, diersoort-iconen opnieuw getekend, mobiele overflow-fix</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>- Echt logo verwerkt
+- Openingstijden per dag getoond
+- Diersoort-iconen opnieuw getekend
+- Mobiele overflow-fix</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr"/>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>25-07-2026</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr"/>
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Van Oosten voor Vis</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr"/>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>24-07-2026</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr"/>
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Zie Haar Stralen</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr"/>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr"/>
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>

<commit_message>
Herinneringen opgevolgd + vaste sjabloon vastgelegd
- follow_up_op = 18-08-2026 voor de 5 bedrijven waaraan Sem een herinneringsmail
  stuurde (Van Oosten, ManiMania, Cone6, Dierenkliniek Animalis, BitWizard).
- Vaste structuur voor herinneringsmails vastgelegd in
  pitches/_HERINNERINGSMAIL_STRUCTUUR.md (altijd deze opmaak gebruiken).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -797,7 +797,11 @@
           <t>nog geen reactie</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>015-2120610</t>
@@ -885,7 +889,11 @@
           <t>nog geen reactie</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
           <t>06 23 774 773</t>
@@ -975,7 +983,11 @@
           <t>nog geen reactie</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
           <t>06 244 606 96</t>
@@ -1066,7 +1078,11 @@
           <t>nog geen reactie</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
           <t>015 737 0135</t>
@@ -1150,7 +1166,11 @@
           <t>nog geen reactie</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
           <t>+31 (0)15-2049110</t>

</xml_diff>

<commit_message>
Feedback Garagebedrijf Dennis (#19) verwerkt: updategeschiedenis + overzicht
Sitefix live (commit b8c7146 in de site-repo, Pages groen). Issue #19 gesloten.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -240,8 +240,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E19" headerRowCount="1">
-  <autoFilter ref="A1:E19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E20" headerRowCount="1">
+  <autoFilter ref="A1:E20"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Datum"/>
@@ -1586,12 +1586,16 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>10-08-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+          <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
+- Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
+- Meta-/verantwoordingstekst over ontbrekende beoordeling verwijderd
+- '10 Google-reviews'-teller weggehaald; kerncijfers nu symmetrisch (38 merken, 6 dagen open)
+- Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1789,105 +1793,109 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Geo B.V.</t>
+          <t>Garagebedrijf Dennis</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr"/>
+          <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
+- Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
+- Meta-/verantwoordingstekst over ontbrekende beoordeling verwijderd
+- '10 Google-reviews'-teller weggehaald; kerncijfers nu symmetrisch (38 merken, 6 dagen open)
+- Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>b8c7146</t>
+        </is>
+      </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/geo/</t>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
           <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>10-08-2026</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
 - Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr"/>
-      <c r="E3" s="9" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Garagebedrijf Dennis</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>10-08-2026</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
       <c r="D4" s="9" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
+      <c r="E4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Smithuis Installatiebedrijf</t>
+          <t>Garagebedrijf Dennis</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>c749bd4</t>
-        </is>
-      </c>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr"/>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Cocon</t>
+          <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1897,24 +1905,24 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>b42a083</t>
+          <t>c749bd4</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Meijer Administratieve Diensten</t>
+          <t>Cocon</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1922,48 +1930,75 @@
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>b42a083</t>
+        </is>
+      </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>30-07-2026</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>- Kaarten op gelijke hoogte gebracht
 - Bannercontrast verbeterd
@@ -1971,29 +2006,29 @@
 - Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>- VetPlan-knop en -disclaimer herzien
 - Contactformulier-melding pas na klik
@@ -2001,36 +2036,9 @@
 - Hamburgermenu-bugs opgelost</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>5ce93c69</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Dierenkliniek Animalis</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>716874d</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2042,7 +2050,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Dierenkliniek Animalis</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -2052,76 +2060,76 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>b576436</t>
+          <t>716874d</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>b576436</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
 - 5 extra foto's opnieuw geplaatst
 - Regio gecorrigeerd</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr"/>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Cone6</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>a5daae7</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Dierenkliniek Animalis</t>
+          <t>Cone6</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -2131,17 +2139,17 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>2c24e39</t>
+          <t>a5daae7</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
@@ -2157,6 +2165,33 @@
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>2c24e39</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>- Echt logo verwerkt
 - Openingstijden per dag getoond
@@ -2164,49 +2199,26 @@
 - Mobiele overflow-fix</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>ManiMania</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>25-07-2026</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr"/>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Van Oosten voor Vis</t>
+          <t>ManiMania</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -2217,19 +2229,19 @@
       <c r="D18" s="9" t="inlineStr"/>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Zie Haar Stralen</t>
+          <t>Van Oosten voor Vis</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -2239,6 +2251,29 @@
       </c>
       <c r="D19" s="9" t="inlineStr"/>
       <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Zie Haar Stralen</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr"/>
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>

<commit_message>
Herinneringsmail-structuur in RULES.md + feedback Meijer (#20) verwerkt
- RULES.md: nieuwe sectie 'Herinneringsmail' met Sems vaste opzet (onderwerp,
  Emailadres-regel, beschrijvende link, bullets, vaste afsluiting).
- Meijer (#20) sitefix live (commit 2ee6bf43, Pages groen): updategeschiedenis
  + overzicht bijgewerkt. Issue #20 gesloten.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -240,8 +240,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E20" headerRowCount="1">
-  <autoFilter ref="A1:E20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E21" headerRowCount="1">
+  <autoFilter ref="A1:E21"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Datum"/>
@@ -1269,12 +1269,16 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Reviews: geen aantal meer genoemd, twee uitgeschreven quotes (Anne Rust, Ruben Provencio Kuijk) met vijf sterren; kale namenlijst verwijderd
+- Achtergrondfoto 'Even sparren over uw administratie?' lichter gemaakt
+- Lettertype sitebreed iets kleiner; Google Maps-kaart even breed maar minder hoog
+- Taalswitcher nu een landendropdown met vlaggen (NL/EN)
+- Contactformulier losgekoppeld van mailto (alleen bevestiging), adressen linken naar Google Maps, footer-lettertype klein en uniform</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1793,15 +1797,46 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
+          <t>Meijer Administratieve Diensten</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>- Reviews: geen aantal meer genoemd, twee uitgeschreven quotes (Anne Rust, Ruben Provencio Kuijk) met vijf sterren; kale namenlijst verwijderd
+- Achtergrondfoto 'Even sparren over uw administratie?' lichter gemaakt
+- Lettertype sitebreed iets kleiner; Google Maps-kaart even breed maar minder hoog
+- Taalswitcher nu een landendropdown met vlaggen (NL/EN)
+- Contactformulier losgekoppeld van mailto (alleen bevestiging), adressen linken naar Google Maps, footer-lettertype klein en uniform</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>2ee6bf43</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
 - Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
@@ -1810,119 +1845,92 @@
 - Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>b8c7146</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Geo B.V.</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>11-08-2026</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr"/>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
           <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>10-08-2026</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
 - Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Garagebedrijf Dennis</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>10-08-2026</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
       <c r="D5" s="9" t="inlineStr"/>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
+      <c r="E5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Smithuis Installatiebedrijf</t>
+          <t>Garagebedrijf Dennis</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>c749bd4</t>
-        </is>
-      </c>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr"/>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Cocon</t>
+          <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1932,24 +1940,24 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>b42a083</t>
+          <t>c749bd4</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Meijer Administratieve Diensten</t>
+          <t>Cocon</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1957,48 +1965,75 @@
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>b42a083</t>
+        </is>
+      </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>30-07-2026</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr"/>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>- Kaarten op gelijke hoogte gebracht
 - Bannercontrast verbeterd
@@ -2006,29 +2041,29 @@
 - Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>- VetPlan-knop en -disclaimer herzien
 - Contactformulier-melding pas na klik
@@ -2036,36 +2071,9 @@
 - Hamburgermenu-bugs opgelost</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>5ce93c69</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Dierenkliniek Animalis</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>716874d</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -2077,7 +2085,7 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Dierenkliniek Animalis</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
@@ -2087,76 +2095,76 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>b576436</t>
+          <t>716874d</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>b576436</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
 - 5 extra foto's opnieuw geplaatst
 - Regio gecorrigeerd</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr"/>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Cone6</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>a5daae7</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Dierenkliniek Animalis</t>
+          <t>Cone6</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -2166,17 +2174,17 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>2c24e39</t>
+          <t>a5daae7</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
@@ -2192,6 +2200,33 @@
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>2c24e39</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>- Echt logo verwerkt
 - Openingstijden per dag getoond
@@ -2199,49 +2234,26 @@
 - Mobiele overflow-fix</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>ManiMania</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>25-07-2026</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr"/>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Van Oosten voor Vis</t>
+          <t>ManiMania</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -2252,19 +2264,19 @@
       <c r="D19" s="9" t="inlineStr"/>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Zie Haar Stralen</t>
+          <t>Van Oosten voor Vis</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2274,6 +2286,29 @@
       </c>
       <c r="D20" s="9" t="inlineStr"/>
       <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Zie Haar Stralen</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr"/>
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>

<commit_message>
Feedback Cocon (#21) verwerkt: pitch bijgewerkt + updategeschiedenis + overzicht
Sitefix live (commit 06bad74 in de site-repo, Pages groen). Conceptmail cocon-b-b
aangepast: operationele framing en uitleg dat details later (of via een CMS)
aanpasbaar zijn. Issue #21 gesloten.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -240,8 +240,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E21" headerRowCount="1">
-  <autoFilter ref="A1:E21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E22" headerRowCount="1">
+  <autoFilter ref="A1:E22"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Datum"/>
@@ -1349,12 +1349,16 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Herzien naar een operationele B&amp;B (framing 'nog zoekende' eruit)
+- Placeholder-/statustekst 'nog even geduld met de details' verwijderd
+- Interactieve SVG-kaart van het Heuvelland met 12 info-markers en toelichtingen eronder
+- Boekingskalender met een paar bezette datums
+- Google Maps-link met pin toegevoegd; conceptmail aangevuld met uitleg over later aanpassen / CMS</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1828,15 +1832,46 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
+          <t>Cocon</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>- Herzien naar een operationele B&amp;B (framing 'nog zoekende' eruit)
+- Placeholder-/statustekst 'nog even geduld met de details' verwijderd
+- Interactieve SVG-kaart van het Heuvelland met 12 info-markers en toelichtingen eronder
+- Boekingskalender met een paar bezette datums
+- Google Maps-link met pin toegevoegd; conceptmail aangevuld met uitleg over later aanpassen / CMS</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>06bad74</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
 - Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
@@ -1845,119 +1880,92 @@
 - Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>b8c7146</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Geo B.V.</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>11-08-2026</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
           <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>10-08-2026</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
 - Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr"/>
-      <c r="E5" s="9" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Garagebedrijf Dennis</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>10-08-2026</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
       <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
+      <c r="E6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Smithuis Installatiebedrijf</t>
+          <t>Garagebedrijf Dennis</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>c749bd4</t>
-        </is>
-      </c>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Cocon</t>
+          <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1967,24 +1975,24 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>b42a083</t>
+          <t>c749bd4</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Meijer Administratieve Diensten</t>
+          <t>Cocon</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1992,48 +2000,75 @@
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>b42a083</t>
+        </is>
+      </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>30-07-2026</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr"/>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>- Kaarten op gelijke hoogte gebracht
 - Bannercontrast verbeterd
@@ -2041,29 +2076,29 @@
 - Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>- VetPlan-knop en -disclaimer herzien
 - Contactformulier-melding pas na klik
@@ -2071,36 +2106,9 @@
 - Hamburgermenu-bugs opgelost</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>5ce93c69</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Dierenkliniek Animalis</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>716874d</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -2112,7 +2120,7 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Dierenkliniek Animalis</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -2122,76 +2130,76 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>b576436</t>
+          <t>716874d</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>b576436</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
 - 5 extra foto's opnieuw geplaatst
 - Regio gecorrigeerd</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr"/>
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Cone6</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>a5daae7</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Dierenkliniek Animalis</t>
+          <t>Cone6</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -2201,17 +2209,17 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>2c24e39</t>
+          <t>a5daae7</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
@@ -2227,6 +2235,33 @@
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>2c24e39</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>- Echt logo verwerkt
 - Openingstijden per dag getoond
@@ -2234,49 +2269,26 @@
 - Mobiele overflow-fix</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>ManiMania</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>25-07-2026</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr"/>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Van Oosten voor Vis</t>
+          <t>ManiMania</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2287,19 +2299,19 @@
       <c r="D20" s="9" t="inlineStr"/>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Zie Haar Stralen</t>
+          <t>Van Oosten voor Vis</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -2309,6 +2321,29 @@
       </c>
       <c r="D21" s="9" t="inlineStr"/>
       <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Zie Haar Stralen</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr"/>
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>

<commit_message>
Feedback Geo (#18) verwerkt: updategeschiedenis + overzicht
Sitefix live (commit c267f89 in de site-repo, Pages groen). Issue #18 gesloten.
Twee openstaande punten voor Sem genoteerd in de issue: exacte catalogi-PDF-URL's
aanleveren, en of ISO/ISCC ook uit de JSON-LD-metadata moet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -240,8 +240,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E22" headerRowCount="1">
-  <autoFilter ref="A1:E22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E23" headerRowCount="1">
+  <autoFilter ref="A1:E23"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Datum"/>
@@ -1738,12 +1738,18 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+          <t>- Logo verder naar links in de header
+- Dienst-iconen allemaal dezelfde kleur
+- 'Wie er bij ons bunkert' nu een lopende balk i.p.v. bulletlijst
+- Foto's volledig zichtbaar gemaakt (geen crop)
+- Certificaten alleen nog op de kwaliteitpagina
+- Footer-lettertype klein en uniform; adressen linken naar Google Maps met pin
+- Contactformulier zonder mailto (met bevestiging); lettertype sitebreed iets kleiner</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1801,15 +1807,48 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>- Logo verder naar links in de header
+- Dienst-iconen allemaal dezelfde kleur
+- 'Wie er bij ons bunkert' nu een lopende balk i.p.v. bulletlijst
+- Foto's volledig zichtbaar gemaakt (geen crop)
+- Certificaten alleen nog op de kwaliteitpagina
+- Footer-lettertype klein en uniform; adressen linken naar Google Maps met pin
+- Contactformulier zonder mailto (met bevestiging); lettertype sitebreed iets kleiner</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>c267f89</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
           <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>- Reviews: geen aantal meer genoemd, twee uitgeschreven quotes (Anne Rust, Ruben Provencio Kuijk) met vijf sterren; kale namenlijst verwijderd
 - Achtergrondfoto 'Even sparren over uw administratie?' lichter gemaakt
@@ -1818,29 +1857,29 @@
 - Contactformulier losgekoppeld van mailto (alleen bevestiging), adressen linken naar Google Maps, footer-lettertype klein en uniform</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>2ee6bf43</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Cocon</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>- Herzien naar een operationele B&amp;B (framing 'nog zoekende' eruit)
 - Placeholder-/statustekst 'nog even geduld met de details' verwijderd
@@ -1849,29 +1888,29 @@
 - Google Maps-link met pin toegevoegd; conceptmail aangevuld met uitleg over later aanpassen / CMS</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>06bad74</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
 - Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
@@ -1880,119 +1919,92 @@
 - Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>b8c7146</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Geo B.V.</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>11-08-2026</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr"/>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
           <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>10-08-2026</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
 - Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Garagebedrijf Dennis</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>10-08-2026</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
       <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
+      <c r="E7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Smithuis Installatiebedrijf</t>
+          <t>Garagebedrijf Dennis</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>c749bd4</t>
-        </is>
-      </c>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Cocon</t>
+          <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -2002,24 +2014,24 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>b42a083</t>
+          <t>c749bd4</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Meijer Administratieve Diensten</t>
+          <t>Cocon</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -2027,48 +2039,75 @@
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>b42a083</t>
+        </is>
+      </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>30-07-2026</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr"/>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>- Kaarten op gelijke hoogte gebracht
 - Bannercontrast verbeterd
@@ -2076,29 +2115,29 @@
 - Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>- VetPlan-knop en -disclaimer herzien
 - Contactformulier-melding pas na klik
@@ -2106,36 +2145,9 @@
 - Hamburgermenu-bugs opgelost</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>5ce93c69</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Dierenkliniek Animalis</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>716874d</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2147,7 +2159,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Dierenkliniek Animalis</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -2157,76 +2169,76 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>b576436</t>
+          <t>716874d</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>b576436</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
 - 5 extra foto's opnieuw geplaatst
 - Regio gecorrigeerd</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr"/>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr"/>
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Cone6</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>a5daae7</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Dierenkliniek Animalis</t>
+          <t>Cone6</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -2236,17 +2248,17 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>2c24e39</t>
+          <t>a5daae7</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
@@ -2262,6 +2274,33 @@
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>2c24e39</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>- Echt logo verwerkt
 - Openingstijden per dag getoond
@@ -2269,49 +2308,26 @@
 - Mobiele overflow-fix</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>ManiMania</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>25-07-2026</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr"/>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Van Oosten voor Vis</t>
+          <t>ManiMania</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -2322,19 +2338,19 @@
       <c r="D21" s="9" t="inlineStr"/>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Zie Haar Stralen</t>
+          <t>Van Oosten voor Vis</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -2344,6 +2360,29 @@
       </c>
       <c r="D22" s="9" t="inlineStr"/>
       <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Zie Haar Stralen</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr"/>
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>

<commit_message>
Schilperoort (#22): companies.json bijgewerkt naar wacht_op_akkoord + overzicht
Status needs_review -> wacht_op_akkoord, live_url en pitch-velden gezet,
updategeschiedenis toegevoegd (de vorige commit miste dit door een scriptfout).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -37,7 +37,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,12 +74,6 @@
         <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
-        <bgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -107,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -128,9 +122,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -240,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E23" headerRowCount="1">
-  <autoFilter ref="A1:E23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E24" headerRowCount="1">
+  <autoFilter ref="A1:E24"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Datum"/>
@@ -1467,9 +1458,9 @@
           <t>Rijswijk</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Needs review</t>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Wacht op akkoord</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1477,13 +1468,17 @@
           <t>schilderpoort-ijzerwaren</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Nee</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
@@ -1510,16 +1505,21 @@
           <t>06-08-2026</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>10-08-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
         <is>
-          <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
-- Niet afgerond; op needs_review gezet</t>
+          <t>- Feedback verwerkt: teksten breder op pc, lettertype iets kleiner, AI-achtige hoofdletters weg, meta-zin bij reviews weg, FAQ-pagina gemoderniseerd, filiaalfoto's op gelijke hoogte
+- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld (met bevestiging), adressen naar Google Maps, diverse fixes
+- Status van needs_review naar wacht_op_akkoord; pitchmail geschreven</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1805,17 +1805,46 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Schilperoort IJzerwaren</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>- Feedback verwerkt: teksten breder op pc, lettertype iets kleiner, AI-achtige hoofdletters weg, meta-zin bij reviews weg, FAQ-pagina gemoderniseerd, filiaalfoto's op gelijke hoogte
+- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld (met bevestiging), adressen naar Google Maps, diverse fixes
+- Status van needs_review naar wacht_op_akkoord; pitchmail geschreven</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>c7fe050</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Geo B.V.</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>20-08-2026</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>- Logo verder naar links in de header
 - Dienst-iconen allemaal dezelfde kleur
@@ -1826,29 +1855,29 @@
 - Contactformulier zonder mailto (met bevestiging); lettertype sitebreed iets kleiner</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>c267f89</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>- Reviews: geen aantal meer genoemd, twee uitgeschreven quotes (Anne Rust, Ruben Provencio Kuijk) met vijf sterren; kale namenlijst verwijderd
 - Achtergrondfoto 'Even sparren over uw administratie?' lichter gemaakt
@@ -1857,29 +1886,29 @@
 - Contactformulier losgekoppeld van mailto (alleen bevestiging), adressen linken naar Google Maps, footer-lettertype klein en uniform</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>2ee6bf43</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Cocon</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>- Herzien naar een operationele B&amp;B (framing 'nog zoekende' eruit)
 - Placeholder-/statustekst 'nog even geduld met de details' verwijderd
@@ -1888,29 +1917,29 @@
 - Google Maps-link met pin toegevoegd; conceptmail aangevuld met uitleg over later aanpassen / CMS</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>06bad74</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
 - Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
@@ -1919,195 +1948,199 @@
 - Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>b8c7146</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Geo B.V.</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>11-08-2026</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>10-08-2026</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
 - Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>10-08-2026</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>04-08-2026</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>c749bd4</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Cocon</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>01-08-2026</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>b42a083</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>31-07-2026</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr"/>
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>BitWizard B.V.</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>30-07-2026</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>- Kaarten op gelijke hoogte gebracht
 - Bannercontrast verbeterd
@@ -2115,29 +2148,29 @@
 - Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>- VetPlan-knop en -disclaimer herzien
 - Contactformulier-melding pas na klik
@@ -2145,162 +2178,162 @@
 - Hamburgermenu-bugs opgelost</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>5ce93c69</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>716874d</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>BitWizard B.V.</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>b576436</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
 - 5 extra foto's opnieuw geplaatst
 - Regio gecorrigeerd</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr"/>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr"/>
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>a5daae7</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>2c24e39</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>- Echt logo verwerkt
 - Openingstijden per dag getoond
@@ -2308,81 +2341,81 @@
 - Mobiele overflow-fix</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>25-07-2026</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr"/>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr"/>
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Van Oosten voor Vis</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>24-07-2026</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr"/>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Zie Haar Stralen</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>23-07-2026</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr"/>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr"/>
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>

<commit_message>
Schilperoort (#22): status afgerond naar wacht_op_akkoord + updategeschiedenis
Vervolg op de eerdere commit (pitchmail stond al klaar): companies.json-update
die door een scriptfout niet was doorgevoerd, nu alsnog: status needs_review ->
wacht_op_akkoord, live_url, pitch_email_klaar, afgerond_op, updates-entry.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E24" headerRowCount="1">
-  <autoFilter ref="A1:E24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E25" headerRowCount="1">
+  <autoFilter ref="A1:E25"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Datum"/>
@@ -1518,7 +1518,7 @@
       <c r="R11" s="6" t="inlineStr">
         <is>
           <t>- Feedback verwerkt: teksten breder op pc, lettertype iets kleiner, AI-achtige hoofdletters weg, meta-zin bij reviews weg, FAQ-pagina gemoderniseerd, filiaalfoto's op gelijke hoogte
-- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld (met bevestiging), adressen naar Google Maps, diverse fixes
+- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld met bevestiging, adressen naar Google Maps, diverse fixes
 - Status van needs_review naar wacht_op_akkoord; pitchmail geschreven</t>
         </is>
       </c>
@@ -1767,7 +1767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1836,15 +1836,44 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
+          <t>Schilperoort IJzerwaren</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>20-08-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>- Feedback verwerkt: teksten breder op pc, lettertype iets kleiner, AI-achtige hoofdletters weg, meta-zin bij reviews weg, FAQ-pagina gemoderniseerd, filiaalfoto's op gelijke hoogte
+- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld met bevestiging, adressen naar Google Maps, diverse fixes
+- Status van needs_review naar wacht_op_akkoord; pitchmail geschreven</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>c7fe050</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
           <t>Geo B.V.</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>20-08-2026</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>- Logo verder naar links in de header
 - Dienst-iconen allemaal dezelfde kleur
@@ -1855,29 +1884,29 @@
 - Contactformulier zonder mailto (met bevestiging); lettertype sitebreed iets kleiner</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>c267f89</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>- Reviews: geen aantal meer genoemd, twee uitgeschreven quotes (Anne Rust, Ruben Provencio Kuijk) met vijf sterren; kale namenlijst verwijderd
 - Achtergrondfoto 'Even sparren over uw administratie?' lichter gemaakt
@@ -1886,29 +1915,29 @@
 - Contactformulier losgekoppeld van mailto (alleen bevestiging), adressen linken naar Google Maps, footer-lettertype klein en uniform</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>2ee6bf43</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Cocon</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>- Herzien naar een operationele B&amp;B (framing 'nog zoekende' eruit)
 - Placeholder-/statustekst 'nog even geduld met de details' verwijderd
@@ -1917,29 +1946,29 @@
 - Google Maps-link met pin toegevoegd; conceptmail aangevuld met uitleg over later aanpassen / CMS</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>06bad74</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
 - Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
@@ -1948,123 +1977,96 @@
 - Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>b8c7146</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Geo B.V.</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>11-08-2026</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr"/>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/geo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
           <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>10-08-2026</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
 - Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr"/>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Garagebedrijf Dennis</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>10-08-2026</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
       <c r="D9" s="8" t="inlineStr"/>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
+          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Smithuis Installatiebedrijf</t>
+          <t>Garagebedrijf Dennis</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>c749bd4</t>
-        </is>
-      </c>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Cocon</t>
+          <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -2074,24 +2076,24 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>b42a083</t>
+          <t>c749bd4</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Meijer Administratieve Diensten</t>
+          <t>Cocon</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -2099,48 +2101,75 @@
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>b42a083</t>
+        </is>
+      </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>30-07-2026</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>30-07-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr"/>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
           <t>Cone6</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>- Kaarten op gelijke hoogte gebracht
 - Bannercontrast verbeterd
@@ -2148,29 +2177,29 @@
 - Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>- VetPlan-knop en -disclaimer herzien
 - Contactformulier-melding pas na klik
@@ -2178,36 +2207,9 @@
 - Hamburgermenu-bugs opgelost</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>5ce93c69</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Dierenkliniek Animalis</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>716874d</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -2219,7 +2221,7 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Dierenkliniek Animalis</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -2229,76 +2231,76 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>b576436</t>
+          <t>716874d</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>BitWizard B.V.</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>b576436</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
           <t>ManiMania</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>27-07-2026</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
 - 5 extra foto's opnieuw geplaatst
 - Regio gecorrigeerd</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr"/>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/manimania/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Cone6</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>a5daae7</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Dierenkliniek Animalis</t>
+          <t>Cone6</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -2308,17 +2310,17 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>2c24e39</t>
+          <t>a5daae7</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
@@ -2334,6 +2336,33 @@
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>2c24e39</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>- Echt logo verwerkt
 - Openingstijden per dag getoond
@@ -2341,49 +2370,26 @@
 - Mobiele overflow-fix</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>ManiMania</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>25-07-2026</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr"/>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Van Oosten voor Vis</t>
+          <t>ManiMania</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>25-07-2026</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -2394,19 +2400,19 @@
       <c r="D23" s="8" t="inlineStr"/>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Zie Haar Stralen</t>
+          <t>Van Oosten voor Vis</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -2416,6 +2422,29 @@
       </c>
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Zie Haar Stralen</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>23-07-2026</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr"/>
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>

<commit_message>
Schilperoort: dubbele afrondingsnotitie/updates definitief ontdubbeld
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvQ9mJKBUrKQejinBEpFtg
</commit_message>
<xml_diff>
--- a/overzicht.xlsx
+++ b/overzicht.xlsx
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E25" headerRowCount="1">
-  <autoFilter ref="A1:E25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Updategeschiedenis" displayName="Updategeschiedenis" ref="A1:E24" headerRowCount="1">
+  <autoFilter ref="A1:E24"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Bedrijfsnaam"/>
     <tableColumn id="2" name="Datum"/>
@@ -1518,7 +1518,7 @@
       <c r="R11" s="6" t="inlineStr">
         <is>
           <t>- Feedback verwerkt: teksten breder op pc, lettertype iets kleiner, AI-achtige hoofdletters weg, meta-zin bij reviews weg, FAQ-pagina gemoderniseerd, filiaalfoto's op gelijke hoogte
-- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld met bevestiging, adressen naar Google Maps, diverse fixes
+- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld (met bevestiging), adressen naar Google Maps, diverse fixes
 - Status van needs_review naar wacht_op_akkoord; pitchmail geschreven</t>
         </is>
       </c>
@@ -1767,7 +1767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1836,7 +1836,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Schilperoort IJzerwaren</t>
+          <t>Geo B.V.</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1845,35 +1845,6 @@
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>- Feedback verwerkt: teksten breder op pc, lettertype iets kleiner, AI-achtige hoofdletters weg, meta-zin bij reviews weg, FAQ-pagina gemoderniseerd, filiaalfoto's op gelijke hoogte
-- Afrondende kwaliteitscontrole (build was ooit onderbroken): contactformulier van mailto losgekoppeld met bevestiging, adressen naar Google Maps, diverse fixes
-- Status van needs_review naar wacht_op_akkoord; pitchmail geschreven</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>c7fe050</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Geo B.V.</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>20-08-2026</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>- Logo verder naar links in de header
 - Dienst-iconen allemaal dezelfde kleur
@@ -1884,29 +1855,29 @@
 - Contactformulier zonder mailto (met bevestiging); lettertype sitebreed iets kleiner</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>c267f89</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>- Reviews: geen aantal meer genoemd, twee uitgeschreven quotes (Anne Rust, Ruben Provencio Kuijk) met vijf sterren; kale namenlijst verwijderd
 - Achtergrondfoto 'Even sparren over uw administratie?' lichter gemaakt
@@ -1915,29 +1886,29 @@
 - Contactformulier losgekoppeld van mailto (alleen bevestiging), adressen linken naar Google Maps, footer-lettertype klein en uniform</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>2ee6bf43</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Cocon</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>19-08-2026</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>- Herzien naar een operationele B&amp;B (framing 'nog zoekende' eruit)
 - Placeholder-/statustekst 'nog even geduld met de details' verwijderd
@@ -1946,29 +1917,29 @@
 - Google Maps-link met pin toegevoegd; conceptmail aangevuld met uitleg over later aanpassen / CMS</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>06bad74</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Garagebedrijf Dennis</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>- Homepage-kop 'Van Audi tot Volvo' vervangen door 'Met auto's van deze merken werken wij'
 - Merkenbalk toont nu de automerk-logo's (twee sporen) in plaats van de namen
@@ -1977,44 +1948,68 @@
 - Lettertypes sitebreed iets kleiner en ontwerp moderner (marquee, oplopende tellers, gestaggerde reveals)</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>b8c7146</t>
         </is>
       </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Geo B.V.</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>11-08-2026</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr"/>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
+          <t>https://svanwijksolutions.github.io/geo/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Geo B.V.</t>
+          <t>Schilperoort IJzerwaren</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
+          <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
+- Niet afgerond; op needs_review gezet</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/geo/</t>
+          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Schilperoort IJzerwaren</t>
+          <t>Garagebedrijf Dennis</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -2024,49 +2019,52 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>- Bouw deels uitgevoerd (3 commits: basis+FAQ+NL/EN, beeldmateriaal, taal/menu-polish)
-- Niet afgerond; op needs_review gezet</t>
+          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr"/>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/schilderpoort-ijzerwaren/</t>
+          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Garagebedrijf Dennis</t>
+          <t>Smithuis Installatiebedrijf</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>10-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet (5 commits, volledige 8-staps QA)</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr"/>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>c749bd4</t>
+        </is>
+      </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/garagebedrijf-dennis/</t>
+          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Smithuis Installatiebedrijf</t>
+          <t>Cocon</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -2076,24 +2074,24 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>c749bd4</t>
+          <t>b42a083</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/smithuis-installatie/</t>
+          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Cocon</t>
+          <t>Meijer Administratieve Diensten</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>31-07-2026</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -2101,75 +2099,48 @@
           <t>- Eerste versie live gezet</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>b42a083</t>
-        </is>
-      </c>
+      <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cocon-b-b/</t>
+          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Meijer Administratieve Diensten</t>
+          <t>BitWizard B.V.</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>31-07-2026</t>
+          <t>30-07-2026</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet</t>
+          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/meijer-administratievediensten-demo/</t>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>Cone6</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>30-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>- Feedbackronde (issue #6) deels verwerkt, afgebroken door weeklimiet; issue blijft open</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr"/>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Cone6</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>28-07-2026</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>- Kaarten op gelijke hoogte gebracht
 - Bannercontrast verbeterd
@@ -2177,29 +2148,29 @@
 - Mailto-verzending hersteld en verboden tekst verwijderd</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>eb2a9c7</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Dierenkliniek Animalis</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>28-07-2026</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>- VetPlan-knop en -disclaimer herzien
 - Contactformulier-melding pas na klik
@@ -2207,9 +2178,36 @@
 - Hamburgermenu-bugs opgelost</t>
         </is>
       </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>5ce93c69</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Dierenkliniek Animalis</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>28-07-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
+        </is>
+      </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>5ce93c69</t>
+          <t>716874d</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -2221,7 +2219,7 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Dierenkliniek Animalis</t>
+          <t>BitWizard B.V.</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -2231,76 +2229,76 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>- Favicon en apple-touch-icon opnieuw gegenereerd uit het echte logo</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>716874d</t>
+          <t>b576436</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>BitWizard B.V.</t>
+          <t>ManiMania</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>28-07-2026</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>b576436</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/bitwizard-demo/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>ManiMania</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>- Echte prijslijst verwerkt in nieuwe prijzen.html
 - 5 extra foto's opnieuw geplaatst
 - Regio gecorrigeerd</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr"/>
+      <c r="D18" s="8" t="inlineStr"/>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Cone6</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>27-07-2026</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>a5daae7</t>
+        </is>
+      </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/manimania/</t>
+          <t>https://svanwijksolutions.github.io/cone6/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Cone6</t>
+          <t>Dierenkliniek Animalis</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -2310,17 +2308,17 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>- Eerste versie live gezet (NL/EN, FAQ, algemene voorwaarden, teambuilding-pagina)</t>
+          <t>- Eerste versie live gezet</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>a5daae7</t>
+          <t>2c24e39</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/cone6/</t>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
         </is>
       </c>
     </row>
@@ -2336,33 +2334,6 @@
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>2c24e39</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Dierenkliniek Animalis</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>27-07-2026</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>- Echt logo verwerkt
 - Openingstijden per dag getoond
@@ -2370,26 +2341,49 @@
 - Mobiele overflow-fix</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>0e586ac</t>
         </is>
       </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>ManiMania</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>25-07-2026</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>- Eerste versie live gezet</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/dierenkliniek-animalis/</t>
+          <t>https://svanwijksolutions.github.io/manimania/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>ManiMania</t>
+          <t>Van Oosten voor Vis</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>25-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -2400,19 +2394,19 @@
       <c r="D23" s="8" t="inlineStr"/>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>https://svanwijksolutions.github.io/manimania/</t>
+          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Van Oosten voor Vis</t>
+          <t>Zie Haar Stralen</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -2422,29 +2416,6 @@
       </c>
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>https://svanwijksolutions.github.io/vanoostenvoorvis/</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Zie Haar Stralen</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>23-07-2026</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>- Eerste versie live gezet</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr"/>
-      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>https://svanwijksolutions.github.io/ziehaarstralen-demo/</t>
         </is>

</xml_diff>